<commit_message>
Add IJESM revision robustness analyses
</commit_message>
<xml_diff>
--- a/outputs/tables/c15_exclusion_outputs.xlsx
+++ b/outputs/tables/c15_exclusion_outputs.xlsx
@@ -7,9 +7,9 @@
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="Table_14_summary" sheetId="1" r:id="rId1"/>
-    <sheet name="Table_S8_full_comparison" sheetId="2" r:id="rId2"/>
-    <sheet name="Table_S9_no_c15_top10" sheetId="3" r:id="rId3"/>
+    <sheet name="Table_15_summary" sheetId="1" r:id="rId1"/>
+    <sheet name="Table_S8_full" sheetId="2" r:id="rId2"/>
+    <sheet name="Table_S9_top10" sheetId="3" r:id="rId3"/>
     <sheet name="Table_S10_deterministic" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3130,7 +3130,7 @@
         <v>22</v>
       </c>
       <c r="E2">
-        <v>0.8759368168895242</v>
+        <v>0.8759368168895243</v>
       </c>
       <c r="F2">
         <v>20</v>
@@ -3150,7 +3150,7 @@
         <v>25</v>
       </c>
       <c r="E3">
-        <v>0.882594135802732</v>
+        <v>0.8825941358027318</v>
       </c>
       <c r="F3">
         <v>22</v>
@@ -3164,13 +3164,13 @@
         <v>49</v>
       </c>
       <c r="C4">
-        <v>0.1215325709832871</v>
+        <v>0.1215325709832872</v>
       </c>
       <c r="D4">
         <v>27</v>
       </c>
       <c r="E4">
-        <v>0.9372187740684708</v>
+        <v>0.9372187740684705</v>
       </c>
       <c r="F4">
         <v>25</v>
@@ -3190,7 +3190,7 @@
         <v>5</v>
       </c>
       <c r="E5">
-        <v>0.4893743272628885</v>
+        <v>0.4893743272628884</v>
       </c>
       <c r="F5">
         <v>3</v>
@@ -3210,7 +3210,7 @@
         <v>11</v>
       </c>
       <c r="E6">
-        <v>0.7546915206678098</v>
+        <v>0.7546915206678095</v>
       </c>
       <c r="F6">
         <v>10</v>
@@ -3230,7 +3230,7 @@
         <v>8</v>
       </c>
       <c r="E7">
-        <v>0.699683520496182</v>
+        <v>0.6996835204961822</v>
       </c>
       <c r="F7">
         <v>7</v>
@@ -3270,7 +3270,7 @@
         <v>12</v>
       </c>
       <c r="E9">
-        <v>0.746061690320635</v>
+        <v>0.7460616903206352</v>
       </c>
       <c r="F9">
         <v>9</v>
@@ -3290,7 +3290,7 @@
         <v>18</v>
       </c>
       <c r="E10">
-        <v>0.8102142900722566</v>
+        <v>0.8102142900722565</v>
       </c>
       <c r="F10">
         <v>13</v>
@@ -3350,7 +3350,7 @@
         <v>13</v>
       </c>
       <c r="E13">
-        <v>0.7901178506735247</v>
+        <v>0.7901178506735246</v>
       </c>
       <c r="F13">
         <v>11</v>
@@ -3510,7 +3510,7 @@
         <v>4</v>
       </c>
       <c r="E21">
-        <v>0.5146187970602142</v>
+        <v>0.5146187970602143</v>
       </c>
       <c r="F21">
         <v>4</v>
@@ -3570,7 +3570,7 @@
         <v>20</v>
       </c>
       <c r="E24">
-        <v>0.828263333568146</v>
+        <v>0.8282633335681457</v>
       </c>
       <c r="F24">
         <v>15</v>
@@ -3610,7 +3610,7 @@
         <v>28</v>
       </c>
       <c r="E26">
-        <v>0.9229966998569304</v>
+        <v>0.9229966998569302</v>
       </c>
       <c r="F26">
         <v>23</v>
@@ -3690,7 +3690,7 @@
         <v>1</v>
       </c>
       <c r="E30">
-        <v>0.4011722539763569</v>
+        <v>0.401172253976357</v>
       </c>
       <c r="F30">
         <v>2</v>

</xml_diff>